<commit_message>
Add multilingual assignment dropdown authoring updates
</commit_message>
<xml_diff>
--- a/templates/Strukturvorlage_DataDictionary_empty_public_v0.9.4.xlsx
+++ b/templates/Strukturvorlage_DataDictionary_empty_public_v0.9.4.xlsx
@@ -20,19 +20,23 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="Base_Type">Rules!$L$2:$L$47</definedName>
-    <definedName name="Beschreibung">Rules!$M$2:$M$47</definedName>
-    <definedName name="Category">Rules!$K$2:$K$47</definedName>
-    <definedName name="DataType">Rules!$I$2:$I$47</definedName>
-    <definedName name="FAIR_Prinzipien">Rules!$P$2:$P$47</definedName>
-    <definedName name="IFC_Data_Type">Rules!$J$2:$J$47</definedName>
-    <definedName name="ISG___Informationssicherheitsgesetz">Rules!$O$2:$O$47</definedName>
+    <definedName name="DataType">'Rules'!$I$2:$I$47</definedName>
+    <definedName name="FAIR_Prinzipien">'Rules'!$M$2:$M$47</definedName>
+    <definedName name="IFC_Data_Type">'Rules'!$J$2:$J$47</definedName>
+    <definedName name="ISG___Informationssicherheitsgesetz">'Rules'!$L$2:$L$47</definedName>
     <definedName name="Klassifikation">Rules!$B$2:$B$47</definedName>
-    <definedName name="LifecycleStatus">Rules!$Q$2:$Q$47</definedName>
+    <definedName name="LifecycleStatus">'Rules'!$N$2:$N$47</definedName>
     <definedName name="Markmals_Klassifikation">Rules!$F$2:$F$47</definedName>
-    <definedName name="Objekt_Einordnung">Rules!$A$2:$A$47</definedName>
-    <definedName name="Property_Classification">Rules!$E$2:$E$47</definedName>
-    <definedName name="Status">Rules!$N$2:$N$47</definedName>
+    <definedName name="Objekt_Einordnung">'Rules'!$A$2:$A$47</definedName>
+    <definedName name="Property_Classification">'Rules'!$E$2:$E$47</definedName>
+    <definedName name="Status">'Rules'!$K$2:$K$47</definedName>
+    <definedName name="Class-Assignment">'Rules'!$A$2:$A$47</definedName>
+    <definedName name="Klassen_Zuordnung">'Rules'!$B$2:$B$47</definedName>
+    <definedName name="Affectation_de_classe">'Rules'!$C$2:$C$47</definedName>
+    <definedName name="Assegnazione_della_classe">'Rules'!$D$2:$D$47</definedName>
+    <definedName name="Merkmals_Zuordnung">'Rules'!$F$2:$F$47</definedName>
+    <definedName name="Attribution_de_propriete">'Rules'!$G$2:$G$47</definedName>
+    <definedName name="Assegnazione_della_proprieta">'Rules'!$H$2:$H$47</definedName>
     <definedName name="Beschreibung" localSheetId="2">Rules!$F$2:$F$47</definedName>
     <definedName name="DataType" localSheetId="2">Rules!$B$2:$B$47</definedName>
     <definedName name="FAIR_Prinzipien" localSheetId="2">Rules!$I$2:$I$47</definedName>
@@ -10946,7 +10950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" style="223" min="1" max="1"/>
@@ -11021,35 +11025,20 @@
       </c>
       <c r="K1" s="190" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="L1" s="190" t="inlineStr">
         <is>
-          <t>Base Type</t>
+          <t>ISG - Informationssicherheitsgesetz</t>
         </is>
       </c>
       <c r="M1" s="190" t="inlineStr">
         <is>
-          <t>Beschreibung</t>
+          <t>FAIR Prinzipien</t>
         </is>
       </c>
       <c r="N1" s="190" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="O1" s="190" t="inlineStr">
-        <is>
-          <t>ISG - Informationssicherheitsgesetz</t>
-        </is>
-      </c>
-      <c r="P1" s="190" t="inlineStr">
-        <is>
-          <t>FAIR Prinzipien</t>
-        </is>
-      </c>
-      <c r="Q1" s="190" t="inlineStr">
         <is>
           <t>LifecycleStatus</t>
         </is>
@@ -11108,31 +11097,20 @@
       </c>
       <c r="K2" s="77" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Preview</t>
         </is>
       </c>
       <c r="L2" s="77" t="inlineStr">
         <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="M2" s="77" t="n"/>
+          <t>nicht klassifiziert</t>
+        </is>
+      </c>
+      <c r="M2" s="77" t="inlineStr">
+        <is>
+          <t>Zugänglich kostenpflichtig</t>
+        </is>
+      </c>
       <c r="N2" s="77" t="inlineStr">
-        <is>
-          <t>Preview</t>
-        </is>
-      </c>
-      <c r="O2" s="77" t="inlineStr">
-        <is>
-          <t>nicht klassifiziert</t>
-        </is>
-      </c>
-      <c r="P2" s="77" t="inlineStr">
-        <is>
-          <t>Zugänglich kostenpflichtig</t>
-        </is>
-      </c>
-      <c r="Q2" s="77" t="inlineStr">
         <is>
           <t>Preview</t>
         </is>
@@ -11191,35 +11169,20 @@
       </c>
       <c r="K3" s="31" t="inlineStr">
         <is>
-          <t>Simple Defined Type</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="L3" s="31" t="inlineStr">
         <is>
-          <t>STRING</t>
+          <t>intern</t>
         </is>
       </c>
       <c r="M3" s="31" t="inlineStr">
         <is>
-          <t>Datum</t>
+          <t>Zugänglich unentgeltlich</t>
         </is>
       </c>
       <c r="N3" s="31" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="O3" s="31" t="inlineStr">
-        <is>
-          <t>intern</t>
-        </is>
-      </c>
-      <c r="P3" s="31" t="inlineStr">
-        <is>
-          <t>Zugänglich unentgeltlich</t>
-        </is>
-      </c>
-      <c r="Q3" s="31" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
@@ -11278,35 +11241,20 @@
       </c>
       <c r="K4" s="77" t="inlineStr">
         <is>
-          <t>Simple Defined Type</t>
+          <t>Inactive</t>
         </is>
       </c>
       <c r="L4" s="77" t="inlineStr">
         <is>
-          <t>STRING</t>
+          <t>sensitiv</t>
         </is>
       </c>
       <c r="M4" s="77" t="inlineStr">
         <is>
-          <t>Datum und Zeit</t>
+          <t>Nicht zugänglich - kostenpflichtig</t>
         </is>
       </c>
       <c r="N4" s="77" t="inlineStr">
-        <is>
-          <t>Inactive</t>
-        </is>
-      </c>
-      <c r="O4" s="77" t="inlineStr">
-        <is>
-          <t>sensitiv</t>
-        </is>
-      </c>
-      <c r="P4" s="77" t="inlineStr">
-        <is>
-          <t>Nicht zugänglich - kostenpflichtig</t>
-        </is>
-      </c>
-      <c r="Q4" s="77" t="inlineStr">
         <is>
           <t>Inactive</t>
         </is>
@@ -11365,35 +11313,20 @@
       </c>
       <c r="K5" s="31" t="inlineStr">
         <is>
-          <t>Simple Defined Type</t>
+          <t>Deprecated</t>
         </is>
       </c>
       <c r="L5" s="31" t="inlineStr">
         <is>
-          <t>STRING</t>
+          <t>geheim</t>
         </is>
       </c>
       <c r="M5" s="31" t="inlineStr">
         <is>
-          <t>Zeitdauer</t>
+          <t>Nicht zugänglich - unentgeltlich</t>
         </is>
       </c>
       <c r="N5" s="31" t="inlineStr">
-        <is>
-          <t>Deprecated</t>
-        </is>
-      </c>
-      <c r="O5" s="31" t="inlineStr">
-        <is>
-          <t>geheim</t>
-        </is>
-      </c>
-      <c r="P5" s="31" t="inlineStr">
-        <is>
-          <t>Nicht zugänglich - unentgeltlich</t>
-        </is>
-      </c>
-      <c r="Q5" s="31" t="inlineStr">
         <is>
           <t>Deprecated</t>
         </is>
@@ -11452,27 +11385,12 @@
       </c>
       <c r="K6" s="77" t="inlineStr">
         <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L6" s="77" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M6" s="77" t="inlineStr">
-        <is>
-          <t>Globale eindeutige ID</t>
-        </is>
-      </c>
+          <t>Retired</t>
+        </is>
+      </c>
+      <c r="L6" s="77" t="n"/>
+      <c r="M6" s="77" t="n"/>
       <c r="N6" s="77" t="inlineStr">
-        <is>
-          <t>Retired</t>
-        </is>
-      </c>
-      <c r="O6" s="77" t="n"/>
-      <c r="P6" s="77" t="n"/>
-      <c r="Q6" s="77" t="inlineStr">
         <is>
           <t>Retired</t>
         </is>
@@ -11531,27 +11449,12 @@
       </c>
       <c r="K7" s="31" t="inlineStr">
         <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L7" s="31" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M7" s="31" t="inlineStr">
-        <is>
-          <t>Eindeutiger Identifikator</t>
-        </is>
-      </c>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="L7" s="31" t="n"/>
+      <c r="M7" s="31" t="n"/>
       <c r="N7" s="31" t="inlineStr">
-        <is>
-          <t>Candidate</t>
-        </is>
-      </c>
-      <c r="O7" s="31" t="n"/>
-      <c r="P7" s="31" t="n"/>
-      <c r="Q7" s="31" t="inlineStr">
         <is>
           <t>Candidate</t>
         </is>
@@ -11610,27 +11513,12 @@
       </c>
       <c r="K8" s="77" t="inlineStr">
         <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L8" s="77" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M8" s="77" t="inlineStr">
-        <is>
-          <t>Ganzzahl</t>
-        </is>
-      </c>
+          <t>Recorded</t>
+        </is>
+      </c>
+      <c r="L8" s="77" t="n"/>
+      <c r="M8" s="77" t="n"/>
       <c r="N8" s="77" t="inlineStr">
-        <is>
-          <t>Recorded</t>
-        </is>
-      </c>
-      <c r="O8" s="77" t="n"/>
-      <c r="P8" s="77" t="n"/>
-      <c r="Q8" s="77" t="inlineStr">
         <is>
           <t>Recorded</t>
         </is>
@@ -11685,27 +11573,12 @@
       </c>
       <c r="K9" s="31" t="inlineStr">
         <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L9" s="31" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M9" s="31" t="inlineStr">
-        <is>
-          <t>Lokale Uhrzeit</t>
-        </is>
-      </c>
+          <t>Superseded</t>
+        </is>
+      </c>
+      <c r="L9" s="31" t="n"/>
+      <c r="M9" s="31" t="n"/>
       <c r="N9" s="31" t="inlineStr">
-        <is>
-          <t>Superseded</t>
-        </is>
-      </c>
-      <c r="O9" s="31" t="n"/>
-      <c r="P9" s="31" t="n"/>
-      <c r="Q9" s="31" t="inlineStr">
         <is>
           <t>Superseded</t>
         </is>
@@ -11744,27 +11617,12 @@
       </c>
       <c r="K10" s="77" t="inlineStr">
         <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L10" s="77" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M10" s="77" t="inlineStr">
-        <is>
-          <t>Logischer Wert</t>
-        </is>
-      </c>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="L10" s="77" t="n"/>
+      <c r="M10" s="77" t="n"/>
       <c r="N10" s="77" t="inlineStr">
-        <is>
-          <t>Incomplete</t>
-        </is>
-      </c>
-      <c r="O10" s="77" t="n"/>
-      <c r="P10" s="77" t="n"/>
-      <c r="Q10" s="77" t="inlineStr">
         <is>
           <t>Incomplete</t>
         </is>
@@ -11801,25 +11659,10 @@
           <t>IfcLengthMeasure</t>
         </is>
       </c>
-      <c r="K11" s="77" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L11" s="77" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M11" s="77" t="inlineStr">
-        <is>
-          <t>Mass für Länge</t>
-        </is>
-      </c>
+      <c r="K11" s="77" t="n"/>
+      <c r="L11" s="77" t="n"/>
+      <c r="M11" s="77" t="n"/>
       <c r="N11" s="77" t="n"/>
-      <c r="O11" s="77" t="n"/>
-      <c r="P11" s="77" t="n"/>
-      <c r="Q11" s="77" t="n"/>
     </row>
     <row r="12" customFormat="1" s="76">
       <c r="A12" s="81" t="n"/>
@@ -11852,25 +11695,10 @@
           <t>IfcLocalTime</t>
         </is>
       </c>
-      <c r="K12" s="31" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L12" s="31" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M12" s="31" t="inlineStr">
-        <is>
-          <t>Positiver Ganzzahlwert</t>
-        </is>
-      </c>
+      <c r="K12" s="31" t="n"/>
+      <c r="L12" s="31" t="n"/>
+      <c r="M12" s="31" t="n"/>
       <c r="N12" s="31" t="n"/>
-      <c r="O12" s="31" t="n"/>
-      <c r="P12" s="31" t="n"/>
-      <c r="Q12" s="31" t="n"/>
     </row>
     <row r="13" customFormat="1" s="76">
       <c r="A13" s="81" t="n"/>
@@ -11903,25 +11731,10 @@
           <t>IfcLogical</t>
         </is>
       </c>
-      <c r="K13" s="77" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L13" s="77" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M13" s="77" t="inlineStr">
-        <is>
-          <t>Positiver Längenwert</t>
-        </is>
-      </c>
+      <c r="K13" s="77" t="n"/>
+      <c r="L13" s="77" t="n"/>
+      <c r="M13" s="77" t="n"/>
       <c r="N13" s="77" t="n"/>
-      <c r="O13" s="77" t="n"/>
-      <c r="P13" s="77" t="n"/>
-      <c r="Q13" s="77" t="n"/>
     </row>
     <row r="14" customFormat="1" s="76">
       <c r="A14" s="81" t="n"/>
@@ -11954,25 +11767,10 @@
           <t>IfcNormalisedRatioMeasure</t>
         </is>
       </c>
-      <c r="K14" s="31" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L14" s="31" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M14" s="31" t="inlineStr">
-        <is>
-          <t>Positiver Verhältniswert</t>
-        </is>
-      </c>
+      <c r="K14" s="31" t="n"/>
+      <c r="L14" s="31" t="n"/>
+      <c r="M14" s="31" t="n"/>
       <c r="N14" s="31" t="n"/>
-      <c r="O14" s="31" t="n"/>
-      <c r="P14" s="31" t="n"/>
-      <c r="Q14" s="31" t="n"/>
     </row>
     <row r="15" customFormat="1" s="76">
       <c r="A15" s="81" t="n"/>
@@ -12005,25 +11803,10 @@
           <t>IfcPositiveInteger</t>
         </is>
       </c>
-      <c r="K15" s="77" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L15" s="77" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M15" s="77" t="inlineStr">
-        <is>
-          <t>Positives Zeitmass</t>
-        </is>
-      </c>
+      <c r="K15" s="77" t="n"/>
+      <c r="L15" s="77" t="n"/>
+      <c r="M15" s="77" t="n"/>
       <c r="N15" s="77" t="n"/>
-      <c r="O15" s="77" t="n"/>
-      <c r="P15" s="77" t="n"/>
-      <c r="Q15" s="77" t="n"/>
     </row>
     <row r="16" customFormat="1" s="76">
       <c r="A16" s="81" t="n"/>
@@ -12056,25 +11839,10 @@
           <t>IfcPositiveLengthMeasure</t>
         </is>
       </c>
-      <c r="K16" s="31" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L16" s="31" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M16" s="31" t="inlineStr">
-        <is>
-          <t>Reelle Zahl</t>
-        </is>
-      </c>
+      <c r="K16" s="31" t="n"/>
+      <c r="L16" s="31" t="n"/>
+      <c r="M16" s="31" t="n"/>
       <c r="N16" s="31" t="n"/>
-      <c r="O16" s="31" t="n"/>
-      <c r="P16" s="31" t="n"/>
-      <c r="Q16" s="31" t="n"/>
     </row>
     <row r="17" customFormat="1" s="76">
       <c r="A17" s="81" t="n"/>
@@ -12107,25 +11875,10 @@
           <t>IfcPositiveRatioMeasure</t>
         </is>
       </c>
-      <c r="K17" s="77" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L17" s="77" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M17" s="77" t="inlineStr">
-        <is>
-          <t>Verhältniswert</t>
-        </is>
-      </c>
+      <c r="K17" s="77" t="n"/>
+      <c r="L17" s="77" t="n"/>
+      <c r="M17" s="77" t="n"/>
       <c r="N17" s="77" t="n"/>
-      <c r="O17" s="77" t="n"/>
-      <c r="P17" s="77" t="n"/>
-      <c r="Q17" s="77" t="n"/>
     </row>
     <row r="18" customFormat="1" s="76">
       <c r="A18" s="81" t="n"/>
@@ -12142,25 +11895,10 @@
           <t>IfcPositiveTimeMeasure</t>
         </is>
       </c>
-      <c r="K18" s="199" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L18" s="199" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M18" s="199" t="inlineStr">
-        <is>
-          <t>Thermischer Transmissionskoeffizient</t>
-        </is>
-      </c>
+      <c r="K18" s="199" t="n"/>
+      <c r="L18" s="199" t="n"/>
+      <c r="M18" s="199" t="n"/>
       <c r="N18" s="199" t="n"/>
-      <c r="O18" s="199" t="n"/>
-      <c r="P18" s="199" t="n"/>
-      <c r="Q18" s="199" t="n"/>
     </row>
     <row r="19" customFormat="1" s="76">
       <c r="A19" s="81" t="n"/>
@@ -12177,25 +11915,10 @@
           <t>IfcRatioMeasure</t>
         </is>
       </c>
-      <c r="K19" s="199" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L19" s="199" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M19" s="199" t="inlineStr">
-        <is>
-          <t>Textwert</t>
-        </is>
-      </c>
+      <c r="K19" s="199" t="n"/>
+      <c r="L19" s="199" t="n"/>
+      <c r="M19" s="199" t="n"/>
       <c r="N19" s="199" t="n"/>
-      <c r="O19" s="199" t="n"/>
-      <c r="P19" s="199" t="n"/>
-      <c r="Q19" s="199" t="n"/>
     </row>
     <row r="20" customFormat="1" s="76">
       <c r="A20" s="81" t="n"/>
@@ -12212,25 +11935,10 @@
           <t>IfcReal</t>
         </is>
       </c>
-      <c r="K20" s="199" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L20" s="199" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M20" s="199" t="inlineStr">
-        <is>
-          <t>Zeitangabe</t>
-        </is>
-      </c>
+      <c r="K20" s="199" t="n"/>
+      <c r="L20" s="199" t="n"/>
+      <c r="M20" s="199" t="n"/>
       <c r="N20" s="199" t="n"/>
-      <c r="O20" s="199" t="n"/>
-      <c r="P20" s="199" t="n"/>
-      <c r="Q20" s="199" t="n"/>
     </row>
     <row r="21" customFormat="1" s="76">
       <c r="A21" s="81" t="n"/>
@@ -12247,25 +11955,10 @@
           <t>IfcText</t>
         </is>
       </c>
-      <c r="K21" s="199" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L21" s="199" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M21" s="199" t="inlineStr">
-        <is>
-          <t>URI-Referenz</t>
-        </is>
-      </c>
+      <c r="K21" s="199" t="n"/>
+      <c r="L21" s="199" t="n"/>
+      <c r="M21" s="199" t="n"/>
       <c r="N21" s="199" t="n"/>
-      <c r="O21" s="199" t="n"/>
-      <c r="P21" s="199" t="n"/>
-      <c r="Q21" s="199" t="n"/>
     </row>
     <row r="22" customFormat="1" s="76">
       <c r="A22" s="81" t="n"/>
@@ -12282,25 +11975,10 @@
           <t>IfcThermalTransmittanceMeasure</t>
         </is>
       </c>
-      <c r="K22" s="199" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L22" s="199" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M22" s="199" t="inlineStr">
-        <is>
-          <t>Wahr/Falsch-Wert</t>
-        </is>
-      </c>
+      <c r="K22" s="199" t="n"/>
+      <c r="L22" s="199" t="n"/>
+      <c r="M22" s="199" t="n"/>
       <c r="N22" s="199" t="n"/>
-      <c r="O22" s="199" t="n"/>
-      <c r="P22" s="199" t="n"/>
-      <c r="Q22" s="199" t="n"/>
     </row>
     <row r="23" customFormat="1" s="76">
       <c r="A23" s="81" t="n"/>
@@ -12317,25 +11995,10 @@
           <t>IfcTime</t>
         </is>
       </c>
-      <c r="K23" s="199" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L23" s="199" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M23" s="199" t="inlineStr">
-        <is>
-          <t>Zeichenwert</t>
-        </is>
-      </c>
+      <c r="K23" s="199" t="n"/>
+      <c r="L23" s="199" t="n"/>
+      <c r="M23" s="199" t="n"/>
       <c r="N23" s="199" t="n"/>
-      <c r="O23" s="199" t="n"/>
-      <c r="P23" s="199" t="n"/>
-      <c r="Q23" s="199" t="n"/>
     </row>
     <row r="24" customFormat="1" s="76">
       <c r="A24" s="81" t="n"/>
@@ -12352,25 +12015,10 @@
           <t>IfcURIReference</t>
         </is>
       </c>
-      <c r="K24" s="199" t="inlineStr">
-        <is>
-          <t>Simple Defined Type</t>
-        </is>
-      </c>
-      <c r="L24" s="199" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="M24" s="199" t="inlineStr">
-        <is>
-          <t>Beschriftung</t>
-        </is>
-      </c>
+      <c r="K24" s="199" t="n"/>
+      <c r="L24" s="199" t="n"/>
+      <c r="M24" s="199" t="n"/>
       <c r="N24" s="199" t="n"/>
-      <c r="O24" s="199" t="n"/>
-      <c r="P24" s="199" t="n"/>
-      <c r="Q24" s="199" t="n"/>
     </row>
     <row r="25" customFormat="1" s="76">
       <c r="A25" s="81" t="n"/>
@@ -12387,9 +12035,6 @@
       <c r="L25" s="199" t="n"/>
       <c r="M25" s="199" t="n"/>
       <c r="N25" s="199" t="n"/>
-      <c r="O25" s="199" t="n"/>
-      <c r="P25" s="199" t="n"/>
-      <c r="Q25" s="199" t="n"/>
     </row>
     <row r="26" customFormat="1" s="76">
       <c r="A26" s="81" t="n"/>
@@ -12406,9 +12051,6 @@
       <c r="L26" s="199" t="n"/>
       <c r="M26" s="199" t="n"/>
       <c r="N26" s="199" t="n"/>
-      <c r="O26" s="199" t="n"/>
-      <c r="P26" s="199" t="n"/>
-      <c r="Q26" s="199" t="n"/>
     </row>
     <row r="27" customFormat="1" s="76">
       <c r="A27" s="81" t="n"/>
@@ -12425,9 +12067,6 @@
       <c r="L27" s="199" t="n"/>
       <c r="M27" s="199" t="n"/>
       <c r="N27" s="199" t="n"/>
-      <c r="O27" s="199" t="n"/>
-      <c r="P27" s="199" t="n"/>
-      <c r="Q27" s="199" t="n"/>
     </row>
     <row r="28" customFormat="1" s="76">
       <c r="A28" s="81" t="n"/>
@@ -12444,9 +12083,6 @@
       <c r="L28" s="199" t="n"/>
       <c r="M28" s="199" t="n"/>
       <c r="N28" s="199" t="n"/>
-      <c r="O28" s="199" t="n"/>
-      <c r="P28" s="199" t="n"/>
-      <c r="Q28" s="199" t="n"/>
     </row>
     <row r="29" customFormat="1" s="76">
       <c r="A29" s="81" t="n"/>
@@ -12463,9 +12099,6 @@
       <c r="L29" s="199" t="n"/>
       <c r="M29" s="199" t="n"/>
       <c r="N29" s="199" t="n"/>
-      <c r="O29" s="199" t="n"/>
-      <c r="P29" s="199" t="n"/>
-      <c r="Q29" s="199" t="n"/>
     </row>
     <row r="30" customFormat="1" s="76">
       <c r="A30" s="81" t="n"/>
@@ -12482,9 +12115,6 @@
       <c r="L30" s="199" t="n"/>
       <c r="M30" s="199" t="n"/>
       <c r="N30" s="199" t="n"/>
-      <c r="O30" s="199" t="n"/>
-      <c r="P30" s="199" t="n"/>
-      <c r="Q30" s="199" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="81" t="n"/>
@@ -12501,9 +12131,6 @@
       <c r="L31" s="199" t="n"/>
       <c r="M31" s="199" t="n"/>
       <c r="N31" s="199" t="n"/>
-      <c r="O31" s="199" t="n"/>
-      <c r="P31" s="199" t="n"/>
-      <c r="Q31" s="199" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="81" t="n"/>
@@ -12520,9 +12147,6 @@
       <c r="L32" s="199" t="n"/>
       <c r="M32" s="199" t="n"/>
       <c r="N32" s="199" t="n"/>
-      <c r="O32" s="199" t="n"/>
-      <c r="P32" s="199" t="n"/>
-      <c r="Q32" s="199" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="81" t="n"/>
@@ -12539,9 +12163,6 @@
       <c r="L33" s="199" t="n"/>
       <c r="M33" s="199" t="n"/>
       <c r="N33" s="199" t="n"/>
-      <c r="O33" s="199" t="n"/>
-      <c r="P33" s="199" t="n"/>
-      <c r="Q33" s="199" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="81" t="n"/>
@@ -12558,9 +12179,6 @@
       <c r="L34" s="199" t="n"/>
       <c r="M34" s="199" t="n"/>
       <c r="N34" s="199" t="n"/>
-      <c r="O34" s="199" t="n"/>
-      <c r="P34" s="199" t="n"/>
-      <c r="Q34" s="199" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="81" t="n"/>
@@ -12577,9 +12195,6 @@
       <c r="L35" s="199" t="n"/>
       <c r="M35" s="199" t="n"/>
       <c r="N35" s="199" t="n"/>
-      <c r="O35" s="199" t="n"/>
-      <c r="P35" s="199" t="n"/>
-      <c r="Q35" s="199" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="81" t="n"/>
@@ -12596,9 +12211,6 @@
       <c r="L36" s="199" t="n"/>
       <c r="M36" s="199" t="n"/>
       <c r="N36" s="199" t="n"/>
-      <c r="O36" s="199" t="n"/>
-      <c r="P36" s="199" t="n"/>
-      <c r="Q36" s="199" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="81" t="n"/>
@@ -12615,9 +12227,6 @@
       <c r="L37" s="199" t="n"/>
       <c r="M37" s="199" t="n"/>
       <c r="N37" s="199" t="n"/>
-      <c r="O37" s="199" t="n"/>
-      <c r="P37" s="199" t="n"/>
-      <c r="Q37" s="199" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="81" t="n"/>
@@ -12634,9 +12243,6 @@
       <c r="L38" s="199" t="n"/>
       <c r="M38" s="199" t="n"/>
       <c r="N38" s="199" t="n"/>
-      <c r="O38" s="199" t="n"/>
-      <c r="P38" s="199" t="n"/>
-      <c r="Q38" s="199" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="81" t="n"/>
@@ -12653,9 +12259,6 @@
       <c r="L39" s="199" t="n"/>
       <c r="M39" s="199" t="n"/>
       <c r="N39" s="199" t="n"/>
-      <c r="O39" s="199" t="n"/>
-      <c r="P39" s="199" t="n"/>
-      <c r="Q39" s="199" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="81" t="n"/>
@@ -12672,9 +12275,6 @@
       <c r="L40" s="199" t="n"/>
       <c r="M40" s="199" t="n"/>
       <c r="N40" s="199" t="n"/>
-      <c r="O40" s="199" t="n"/>
-      <c r="P40" s="199" t="n"/>
-      <c r="Q40" s="199" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="81" t="n"/>
@@ -12691,9 +12291,6 @@
       <c r="L41" s="199" t="n"/>
       <c r="M41" s="199" t="n"/>
       <c r="N41" s="199" t="n"/>
-      <c r="O41" s="199" t="n"/>
-      <c r="P41" s="199" t="n"/>
-      <c r="Q41" s="199" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="81" t="n"/>
@@ -12710,9 +12307,6 @@
       <c r="L42" s="199" t="n"/>
       <c r="M42" s="199" t="n"/>
       <c r="N42" s="199" t="n"/>
-      <c r="O42" s="199" t="n"/>
-      <c r="P42" s="199" t="n"/>
-      <c r="Q42" s="199" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="81" t="n"/>
@@ -12729,9 +12323,6 @@
       <c r="L43" s="199" t="n"/>
       <c r="M43" s="199" t="n"/>
       <c r="N43" s="199" t="n"/>
-      <c r="O43" s="199" t="n"/>
-      <c r="P43" s="199" t="n"/>
-      <c r="Q43" s="199" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="81" t="n"/>
@@ -12748,9 +12339,6 @@
       <c r="L44" s="199" t="n"/>
       <c r="M44" s="199" t="n"/>
       <c r="N44" s="199" t="n"/>
-      <c r="O44" s="199" t="n"/>
-      <c r="P44" s="199" t="n"/>
-      <c r="Q44" s="199" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="81" t="n"/>
@@ -12767,9 +12355,6 @@
       <c r="L45" s="199" t="n"/>
       <c r="M45" s="199" t="n"/>
       <c r="N45" s="199" t="n"/>
-      <c r="O45" s="199" t="n"/>
-      <c r="P45" s="199" t="n"/>
-      <c r="Q45" s="199" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="81" t="n"/>
@@ -12786,9 +12371,6 @@
       <c r="L46" s="199" t="n"/>
       <c r="M46" s="199" t="n"/>
       <c r="N46" s="199" t="n"/>
-      <c r="O46" s="199" t="n"/>
-      <c r="P46" s="199" t="n"/>
-      <c r="Q46" s="199" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="81" t="n"/>
@@ -12805,9 +12387,6 @@
       <c r="L47" s="199" t="n"/>
       <c r="M47" s="199" t="n"/>
       <c r="N47" s="199" t="n"/>
-      <c r="O47" s="199" t="n"/>
-      <c r="P47" s="199" t="n"/>
-      <c r="Q47" s="199" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7086614173228347" right="0.7086614173228347" top="0.7874015748031497" bottom="0.7874015748031497" header="0.3149606299212598" footer="0.3149606299212598"/>
@@ -17115,18 +16694,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="C12" s="231" t="inlineStr">
-        <is>
-          <t>Guide</t>
-        </is>
-      </c>
-      <c r="D12" s="225" t="inlineStr">
-        <is>
-          <t>Private organisations may keep only this tab and delete Dictionary_public.</t>
-        </is>
-      </c>
-    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="232" t="inlineStr">
         <is>
@@ -19325,18 +18893,24 @@
       <c r="AI25" s="54" t="n"/>
     </row>
   </sheetData>
-  <dataValidations xWindow="1091" yWindow="456" count="4">
-    <dataValidation sqref="K2 K3 K4 K5 K6 K7 K8 K9 K10 K11 K12 K13 K14 K15 K16 K17 K18 K19 K20 K21 K22 K23 K24 K25 K26 K27 K28 K29 K30 K31 K32 K33 K34 K35 K36 K37 K38 K39 K40 K41 K42 K43 K44 K45 K46 K47 K48 K49 K50 K51 K52 K53 K54 K55 K56 K57 K58 K59 K60 K61 K62 K63 K64 K65 K66 K67 K68 K69 K70 K71 K72 K73 K74 K75 K76 K77 K78 K79 K80 K81 K82 K83 K84 K85 K86 K87 K88 K89 K90 K91 K92 K93 K94 K95 K96 K97 K98 K99 K100 K101 K102 K103 K104 K105 K106 K107 K108 K109 K110 K111 K112 K113 K114 K115 K116 K117 K118 K119 K120 K121 K122 K123 K124 K125 K126 K127 K128 K129 K130 K131 K132 K133 K134 K135 K136 K137 K138 K139 K140 K141 K142 K143 K144 K145 K146 K147 K148 K149 K150 K151 K152 K153 K154 K155 K156 K157 K158 K159 K160 K161 K162 K163 K164 K165 K166 K167 K168 K169 K170 K171 K172 K173 K174 K175 K176 K177 K178 K179 K180 K181 K182 K183 K184 K185 K186 K187 K188 K189 K190 K191 K192 K193 K194 K195 K196 K197 K198 K199 K200 K201 K202 K203 K204 K205 K206 K207 K208 K209 K210 K211 K212 K213 K214 K215 K216 K217 K218 K219 K220 K221 K222 K223 K224 K225 K226 K227 K228 K229 K230 K231 K232 K233 K234 K235 K236 K237 K238 K239 K240 K241 K242 K243 K244 K245 K246 K247 K248 K249 K250 K251 K252 K253 K254 K255 K256 K257 K258 K259 K260 K261 K262 K263 K264 K265 K266 K267 K268 K269 K270 K271 K272 K273 K274 K275 K276 K277 K278 K279 K280 K281 K282 K283 K284 K285 K286 K287 K288 K289 K290 K291 K292 K293 K294 K295 K296 K297 K298 K299 K300 K301 K302 K303 K304 K305 K306 K307 K308 K309 K310 K311 K312 K313 K314 K315 K316 K317 K318 K319 K320 K321 K322 K323 K324 K325 K326 K327 K328 K329 K330 K331 K332 K333 K334 K335 K336 K337 K338 K339 K340 K341 K342 K343 K344 K345 K346 K347 K348 K349 K350 K351 K352 K353 K354 K355 K356 K357 K358 K359 K360 K361 K362 K363 K364 K365 K366 K367 K368 K369 K370 K371 K372 K373 K374 K375 K376 K377 K378 K379 K380 K381 K382 K383 K384 K385 K386 K387 K388 K389 K390 K391 K392 K393 K394 K395 K396 K397 K398 K399 K400 K401 K402 K403 K404 K405 K406 K407 K408 K409 K410 K411 K412 K413 K414 K415 K416 K417 K418 K419 K420 K421 K422 K423 K424 K425 K426 K427 K428 K429 K430 K431 K432 K433 K434 K435 K436 K437 K438 K439 K440 K441 K442 K443 K444 K445 K446 K447 K448 K449 K450 K451 K452 K453 K454 K455 K456 K457 K458 K459 K460 K461 K462 K463 K464 K465 K466 K467 K468 K469 K470 K471 K472 K473 K474 K475 K476 K477 K478 K479 K480 K481 K482 K483 K484 K485 K486 K487 K488 K489 K490 K491 K492 K493 K494 K495 K496 K497 K498 K499 K500 K501 K502 K503 K504 K505 K506 K507 K508 K509 K510 K511 K512 K513 K514 K515 K516 K517 K518 K519 K520 K521 K522 K523 K524 K525 K526 K527 K528 K529 K530 K531 K532 K533 K534 K535 K536 K537 K538 K539 K540 K541 K542 K543 K544 K545 K546 K547 K548 K549 K550 K551 K552 K553 K554 K555 K556 K557 K558 K559 K560 K561 K562 K563 K564 K565 K566 K567 K568 K569 K570 K571 K572 K573 K574 K575 K576 K577 K578 K579 K580 K581 K582 K583 K584 K585 K586 K587 K588 K589 K590 K591 K592 K593 K594 K595 K596 K597 K598 K599 K600 K601 K602 K603 K604 K605 K606 K607 K608 K609 K610 K611 K612 K613 K614 K615 K616 K617 K618 K619 K620 K621 K622 K623 K624 K625 K626 K627 K628 K629 K630 K631 K632 K633 K634 K635 K636 K637 K638 K639 K640 K641 K642 K643 K644 K645 K646 K647 K648 K649 K650 K651 K652 K653 K654 K655 K656 K657 K658 K659 K660 K661 K662 K663 K664 K665 K666 K667 K668 K669 K670 K671 K672 K673 K674 K675 K676 K677 K678 K679 K680 K681 K682 K683 K684 K685 K686 K687 K688 K689 K690 K691 K692 K693 K694 K695 K696 K697 K698 K699 K700 K701 K702 K703 K704 K705 K706 K707 K708 K709 K710 K711 K712 K713 K714 K715 K716 K717 K718 K719 K720 K721 K722 K723 K724 K725 K726 K727 K728 K729 K730 K731 K732 K733 K734 K735 K736 K737 K738 K739 K740 K741 K742 K743 K744 K745 K746 K747 K748 K749 K750 K751 K752 K753 K754 K755 K756 K757 K758 K759 K760 K761 K762 K763 K764 K765 K766 K767 K768 K769 K770 K771 K772 K773 K774 K775 K776 K777 K778 K779 K780 K781 K782 K783 K784 K785 K786 K787 K788 K789 K790 K791 K792 K793 K794 K795 K796 K797 K798 K799 K800 K801 K802 K803 K804 K805 K806 K807 K808 K809 K810 K811 K812 K813 K814 K815 K816 K817 K818 K819 K820 K821 K822 K823 K824 K825 K826 K827 K828 K829 K830 K831 K832 K833 K834 K835 K836 K837 K838 K839 K840 K841 K842 K843 K844 K845 K846 K847 K848 K849 K850 K851 K852 K853 K854 K855 K856 K857 K858 K859 K860 K861 K862 K863 K864 K865 K866 K867 K868 K869 K870 K871 K872 K873 K874 K875 K876 K877 K878 K879 K880 K881 K882 K883 K884 K885 K886 K887 K888 K889 K890 K891 K892 K893 K894 K895 K896 K897 K898 K899 K900 K901 K902 K903 K904 K905 K906 K907 K908 K909 K910 K911 K912 K913 K914 K915 K916 K917 K918 K919 K920 K921 K922 K923 K924 K925 K926 K927 K928 K929 K930 K931 K932 K933 K934 K935 K936 K937 K938 K939 K940 K941 K942 K943 K944 K945 K946 K947 K948 K949 K950 K951 K952 K953 K954 K955 K956 K957 K958 K959 K960 K961 K962 K963 K964 K965 K966 K967 K968 K969 K970 K971 K972 K973 K974 K975 K976 K977 K978 K979 K980 K981 K982 K983 K984 K985 K986 K987 K988 K989 K990 K991 K992 K993 K994 K995 K996 K997 K998 K999 K1000 K1001 K1002 K1003 K1004 K1005 K1006 K1007 K1008 K1009 K1010 K1011 K1012 K1013 K1014 K1015 K1016 K1017 K1018 K1019 K1020 K1021 K1022 K1023 K1024 K1025 K1026 K1027 K1028 K1029 K1030 K1031 K1032 K1033 K1034 K1035 K1036 K1037 K1038 K1039 K1040 K1041 K1042 K1043 K1044 K1045 K1046 K1047 K1048 K1049 K1050 K1051 K1052 K1053 K1054 K1055 K1056 K1057 K1058 K1059 K1060 K1061 K1062 K1063 K1064 K1065 K1066 K1067 K1068 K1069 K1070 K1071 K1072 K1073 K1074 K1075 K1076 K1077 K1078 K1079 K1080 K1081 K1082 K1083 K1084 K1085 K1086 K1087 K1088 K1089 K1090 K1091 K1092 K1093 K1094 K1095 K1096 K1097 K1098 K1099 K1100 K1101 K1102 K1103 K1104 K1105 K1106 K1107 K1108 K1109 K1110 K1111 K1112 K1113 K1114 K1115 K1116 K1117 K1118 K1119 K1120 K1121 K1122 K1123 K1124 K1125 K1126 K1127 K1128 K1129 K1130 K1131 K1132 K1133 K1134 K1135 K1136 K1137 K1138 K1139 K1140 K1141 K1142 K1143 K1144 K1145 K1146 K1147 K1148 K1149 K1150 K1151 K1152 K1153 K1154 K1155 K1156 K1157 K1158 K1159 K1160 K1161 K1162 K1163 K1164 K1165 K1166 K1167 K1168 K1169 K1170 K1171 K1172 K1173 K1174 K1175 K1176 K1177 K1178 K1179 K1180 K1181 K1182 K1183 K1184 K1185 K1186 K1187 K1188 K1189 K1190 K1191 K1192 K1193 K1194 K1195 K1196 K1197 K1198 K1199 K1200 K1201 K1202 K1203 K1204 K1205 K1206 K1207 K1208 K1209 K1210 K1211 K1212 K1213 K1214 K1215 K1216 K1217 K1218 K1219 K1220 K1221 K1222 K1223 K1224 K1225 K1226 K1227 K1228 K1229 K1230 K1231 K1232 K1233 K1234 K1235 K1236 K1237 K1238 K1239 K1240 K1241 K1242 K1243 K1244 K1245 K1246 K1247 K1248 K1249 K1250 K1251 K1252 K1253 K1254 K1255 K1256 K1257 K1258 K1259 K1260 K1261 K1262 K1263 K1264 K1265 K1266 K1267 K1268 K1269 K1270 K1271 K1272 K1273 K1274 K1275 K1276 K1277 K1278 K1279 K1280 K1281 K1282 K1283 K1284 K1285 K1286 K1287 K1288 K1289 K1290 K1291 K1292 K1293 K1294 K1295 K1296 K1297 K1298 K1299 K1300 K1301 K1302 K1303 K1304 K1305 K1306 K1307 K1308 K1309 K1310 K1311 K1312 K1313 K1314 K1315 K1316 K1317 K1318 K1319 K1320 K1321 K1322 K1323 K1324 K1325 K1326 K1327 K1328 K1329 K1330 K1331 K1332 K1333 K1334 K1335 K1336 K1337 K1338 K1339 K1340 K1341 K1342 K1343 K1344 K1345 K1346 K1347 K1348 K1349 K1350 K1351 K1352 K1353 K1354 K1355 K1356 K1357 K1358 K1359 K1360 K1361 K1362 K1363 K1364 K1365 K1366 K1367 K1368 K1369 K1370 K1371 K1372 K1373 K1374 K1375 K1376 K1377 K1378 K1379 K1380 K1381 K1382 K1383 K1384 K1385 K1386 K1387 K1388 K1389 K1390 K1391 K1392 K1393 K1394 K1395 K1396 K1397 K1398 K1399 K1400 K1401 K1402 K1403 K1404 K1405 K1406 K1407 K1408 K1409 K1410 K1411 K1412 K1413 K1414 K1415 K1416 K1417 K1418 K1419 K1420 K1421 K1422 K1423 K1424 K1425 K1426 K1427 K1428 K1429 K1430 K1431 K1432 K1433 K1434 K1435 K1436 K1437 K1438 K1439 K1440 K1441 K1442 K1443 K1444 K1445 K1446 K1447 K1448 K1449 K1450 K1451 K1452 K1453 K1454 K1455 K1456 K1457 K1458 K1459 K1460 K1461 K1462 K1463 K1464 K1465 K1466 K1467 K1468 K1469 K1470 K1471 K1472 K1473 K1474 K1475 K1476 K1477 K1478 K1479 K1480 K1481 K1482 K1483 K1484 K1485 K1486 K1487 K1488 K1489 K1490 K1491 K1492 K1493 K1494 K1495 K1496 K1497 K1498 K1499 K1500 K1501 K1502 K1503 K1504 K1505 K1506 K1507 K1508 K1509 K1510 K1511 K1512 K1513 K1514 K1515 K1516 K1517 K1518 K1519 K1520 K1521 K1522 K1523 K1524 K1525 K1526 K1527 K1528 K1529 K1530 K1531 K1532 K1533 K1534 K1535 K1536 K1537 K1538 K1539 K1540 K1541 K1542 K1543 K1544 K1545 K1546 K1547 K1548 K1549 K1550 K1551 K1552 K1553 K1554 K1555 K1556 K1557 K1558 K1559 K1560 K1561 K1562 K1563 K1564 K1565 K1566 K1567 K1568 K1569 K1570 K1571 K1572 K1573 K1574 K1575 K1576 K1577 K1578 K1579 K1580 K1581 K1582 K1583 K1584 K1585 K1586 K1587 K1588 K1589 K1590 K1591 K1592 K1593 K1594 K1595 K1596 K1597 K1598 K1599 K1600 K1601 K1602 K1603 K1604 K1605 K1606 K1607 K1608 K1609 K1610 K1611 K1612 K1613 K1614 K1615 K1616 K1617 K1618 K1619 K1620 K1621 K1622 K1623 K1624 K1625 K1626 K1627 K1628 K1629 K1630 K1631 K1632 K1633 K1634 K1635 K1636 K1637 K1638 K1639 K1640 K1641 K1642 K1643 K1644 K1645 K1646 K1647 K1648 K1649 K1650 K1651 K1652 K1653 K1654 K1655 K1656 K1657 K1658 K1659 K1660 K1661 K1662 K1663 K1664 K1665 K1666 K1667 K1668 K1669 K1670 K1671 K1672 K1673 K1674 K1675 K1676 K1677 K1678 K1679 K1680 K1681 K1682 K1683 K1684 K1685 K1686 K1687 K1688 K1689 K1690 K1691 K1692 K1693 K1694 K1695 K1696 K1697 K1698 K1699 K1700 K1701 K1702 K1703 K1704 K1705 K1706 K1707 K1708 K1709 K1710 K1711 K1712 K1713 K1714 K1715 K1716 K1717 K1718 K1719 K1720 K1721 K1722 K1723 K1724 K1725 K1726 K1727 K1728 K1729 K1730 K1731 K1732 K1733 K1734 K1735 K1736 K1737 K1738 K1739 K1740 K1741 K1742 K1743 K1744 K1745 K1746 K1747 K1748 K1749 K1750 K1751 K1752 K1753 K1754 K1755 K1756 K1757 K1758 K1759 K1760 K1761 K1762 K1763 K1764 K1765 K1766 K1767 K1768 K1769 K1770 K1771 K1772 K1773 K1774 K1775 K1776 K1777 K1778 K1779 K1780 K1781 K1782 K1783 K1784 K1785 K1786 K1787 K1788 K1789 K1790 K1791 K1792 K1793 K1794 K1795 K1796 K1797 K1798 K1799 K1800 K1801 K1802 K1803 K1804 K1805 K1806 K1807 K1808 K1809 K1810 K1811 K1812 K1813 K1814 K1815 K1816 K1817 K1818 K1819 K1820 K1821 K1822 K1823 K1824 K1825 K1826 K1827 K1828 K1829 K1830 K1831 K1832 K1833 K1834 K1835 K1836 K1837 K1838 K1839 K1840 K1841 K1842 K1843 K1844 K1845 K1846 K1847 K1848 K1849 K1850 K1851 K1852 K1853 K1854 K1855 K1856 K1857 K1858 K1859 K1860 K1861 K1862 K1863 K1864 K1865 K1866 K1867 K1868 K1869 K1870 K1871 K1872 K1873 K1874 K1875 K1876 K1877 K1878 K1879 K1880 K1881 K1882 K1883 K1884 K1885 K1886 K1887 K1888 K1889 K1890 K1891 K1892 K1893 K1894 K1895 K1896 K1897 K1898 K1899 K1900 K1901 K1902 K1903 K1904 K1905 K1906 K1907 K1908 K1909 K1910 K1911 K1912 K1913 K1914 K1915 K1916 K1917 K1918 K1919 K1920 K1921 K1922 K1923 K1924 K1925 K1926 K1927 K1928 K1929 K1930 K1931 K1932 K1933 K1934 K1935 K1936 K1937 K1938 K1939 K1940 K1941 K1942 K1943 K1944 K1945 K1946 K1947 K1948 K1949 K1950 K1951 K1952 K1953 K1954 K1955 K1956 K1957 K1958 K1959 K1960 K1961 K1962 K1963 K1964 K1965 K1966 K1967 K1968 K1969 K1970 K1971 K1972 K1973 K1974 K1975 K1976 K1977 K1978 K1979 K1980 K1981 K1982 K1983 K1984 K1985 K1986 K1987 K1988 K1989 K1990 K1991 K1992 K1993 K1994 K1995 K1996 K1997 K1998 K1999 K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Objekt_Einordnung</formula1>
-    </dataValidation>
+  <dataValidations xWindow="1091" yWindow="456" count="6">
     <dataValidation sqref="AB8 AB9 AB10 AB11 AB12 AB13 AB14 AB15 AB16 AB17 AB18 AB19 AB20 AB21 AB22 AB23 AB24 AB25 AB26 AB27 AB28 AB29 AB30 AB31 AB32 AB33 AB34 AB35 AB36 AB37 AB38 AB39 AB40 AB41 AB42 AB43 AB44 AB45 AB46 AB47 AB48 AB49 AB50 AB51 AB52 AB53 AB54 AB55 AB56 AB57 AB58 AB59 AB60 AB61 AB62 AB63 AB64 AB65 AB66 AB67 AB68 AB69 AB70 AB71 AB72 AB73 AB74 AB75 AB76 AB77 AB78 AB79 AB80 AB81 AB82 AB83 AB84 AB85 AB86 AB87 AB88 AB89 AB90 AB91 AB92 AB93 AB94 AB95 AB96 AB97 AB98 AB99 AB100 AB101 AB102 AB103 AB104 AB105 AB106 AB107 AB108 AB109 AB110 AB111 AB112 AB113 AB114 AB115 AB116 AB117 AB118 AB119 AB120 AB121 AB122 AB123 AB124 AB125 AB126 AB127 AB128 AB129 AB130 AB131 AB132 AB133 AB134 AB135 AB136 AB137 AB138 AB139 AB140 AB141 AB142 AB143 AB144 AB145 AB146 AB147 AB148 AB149 AB150 AB151 AB152 AB153 AB154 AB155 AB156 AB157 AB158 AB159 AB160 AB161 AB162 AB163 AB164 AB165 AB166 AB167 AB168 AB169 AB170 AB171 AB172 AB173 AB174 AB175 AB176 AB177 AB178 AB179 AB180 AB181 AB182 AB183 AB184 AB185 AB186 AB187 AB188 AB189 AB190 AB191 AB192 AB193 AB194 AB195 AB196 AB197 AB198 AB199 AB200 AB201 AB202 AB203 AB204 AB205 AB206 AB207 AB208 AB209 AB210 AB211 AB212 AB213 AB214 AB215 AB216 AB217 AB218 AB219 AB220 AB221 AB222 AB223 AB224 AB225 AB226 AB227 AB228 AB229 AB230 AB231 AB232 AB233 AB234 AB235 AB236 AB237 AB238 AB239 AB240 AB241 AB242 AB243 AB244 AB245 AB246 AB247 AB248 AB249 AB250 AB251 AB252 AB253 AB254 AB255 AB256 AB257 AB258 AB259 AB260 AB261 AB262 AB263 AB264 AB265 AB266 AB267 AB268 AB269 AB270 AB271 AB272 AB273 AB274 AB275 AB276 AB277 AB278 AB279 AB280 AB281 AB282 AB283 AB284 AB285 AB286 AB287 AB288 AB289 AB290 AB291 AB292 AB293 AB294 AB295 AB296 AB297 AB298 AB299 AB300 AB301 AB302 AB303 AB304 AB305 AB306 AB307 AB308 AB309 AB310 AB311 AB312 AB313 AB314 AB315 AB316 AB317 AB318 AB319 AB320 AB321 AB322 AB323 AB324 AB325 AB326 AB327 AB328 AB329 AB330 AB331 AB332 AB333 AB334 AB335 AB336 AB337 AB338 AB339 AB340 AB341 AB342 AB343 AB344 AB345 AB346 AB347 AB348 AB349 AB350 AB351 AB352 AB353 AB354 AB355 AB356 AB357 AB358 AB359 AB360 AB361 AB362 AB363 AB364 AB365 AB366 AB367 AB368 AB369 AB370 AB371 AB372 AB373 AB374 AB375 AB376 AB377 AB378 AB379 AB380 AB381 AB382 AB383 AB384 AB385 AB386 AB387 AB388 AB389 AB390 AB391 AB392 AB393 AB394 AB395 AB396 AB397 AB398 AB399 AB400 AB401 AB402 AB403 AB404 AB405 AB406 AB407 AB408 AB409 AB410 AB411 AB412 AB413 AB414 AB415 AB416 AB417 AB418 AB419 AB420 AB421 AB422 AB423 AB424 AB425 AB426 AB427 AB428 AB429 AB430 AB431 AB432 AB433 AB434 AB435 AB436 AB437 AB438 AB439 AB440 AB441 AB442 AB443 AB444 AB445 AB446 AB447 AB448 AB449 AB450 AB451 AB452 AB453 AB454 AB455 AB456 AB457 AB458 AB459 AB460 AB461 AB462 AB463 AB464 AB465 AB466 AB467 AB468 AB469 AB470 AB471 AB472 AB473 AB474 AB475 AB476 AB477 AB478 AB479 AB480 AB481 AB482 AB483 AB484 AB485 AB486 AB487 AB488 AB489 AB490 AB491 AB492 AB493 AB494 AB495 AB496 AB497 AB498 AB499 AB500 AB501 AB502 AB503 AB504 AB505 AB506 AB507 AB508 AB509 AB510 AB511 AB512 AB513 AB514 AB515 AB516 AB517 AB518 AB519 AB520 AB521 AB522 AB523 AB524 AB525 AB526 AB527 AB528 AB529 AB530 AB531 AB532 AB533 AB534 AB535 AB536 AB537 AB538 AB539 AB540 AB541 AB542 AB543 AB544 AB545 AB546 AB547 AB548 AB549 AB550 AB551 AB552 AB553 AB554 AB555 AB556 AB557 AB558 AB559 AB560 AB561 AB562 AB563 AB564 AB565 AB566 AB567 AB568 AB569 AB570 AB571 AB572 AB573 AB574 AB575 AB576 AB577 AB578 AB579 AB580 AB581 AB582 AB583 AB584 AB585 AB586 AB587 AB588 AB589 AB590 AB591 AB592 AB593 AB594 AB595 AB596 AB597 AB598 AB599 AB600 AB601 AB602 AB603 AB604 AB605 AB606 AB607 AB608 AB609 AB610 AB611 AB612 AB613 AB614 AB615 AB616 AB617 AB618 AB619 AB620 AB621 AB622 AB623 AB624 AB625 AB626 AB627 AB628 AB629 AB630 AB631 AB632 AB633 AB634 AB635 AB636 AB637 AB638 AB639 AB640 AB641 AB642 AB643 AB644 AB645 AB646 AB647 AB648 AB649 AB650 AB651 AB652 AB653 AB654 AB655 AB656 AB657 AB658 AB659 AB660 AB661 AB662 AB663 AB664 AB665 AB666 AB667 AB668 AB669 AB670 AB671 AB672 AB673 AB674 AB675 AB676 AB677 AB678 AB679 AB680 AB681 AB682 AB683 AB684 AB685 AB686 AB687 AB688 AB689 AB690 AB691 AB692 AB693 AB694 AB695 AB696 AB697 AB698 AB699 AB700 AB701 AB702 AB703 AB704 AB705 AB706 AB707 AB708 AB709 AB710 AB711 AB712 AB713 AB714 AB715 AB716 AB717 AB718 AB719 AB720 AB721 AB722 AB723 AB724 AB725 AB726 AB727 AB728 AB729 AB730 AB731 AB732 AB733 AB734 AB735 AB736 AB737 AB738 AB739 AB740 AB741 AB742 AB743 AB744 AB745 AB746 AB747 AB748 AB749 AB750 AB751 AB752 AB753 AB754 AB755 AB756 AB757 AB758 AB759 AB760 AB761 AB762 AB763 AB764 AB765 AB766 AB767 AB768 AB769 AB770 AB771 AB772 AB773 AB774 AB775 AB776 AB777 AB778 AB779 AB780 AB781 AB782 AB783 AB784 AB785 AB786 AB787 AB788 AB789 AB790 AB791 AB792 AB793 AB794 AB795 AB796 AB797 AB798 AB799 AB800 AB801 AB802 AB803 AB804 AB805 AB806 AB807 AB808 AB809 AB810 AB811 AB812 AB813 AB814 AB815 AB816 AB817 AB818 AB819 AB820 AB821 AB822 AB823 AB824 AB825 AB826 AB827 AB828 AB829 AB830 AB831 AB832 AB833 AB834 AB835 AB836 AB837 AB838 AB839 AB840 AB841 AB842 AB843 AB844 AB845 AB846 AB847 AB848 AB849 AB850 AB851 AB852 AB853 AB854 AB855 AB856 AB857 AB858 AB859 AB860 AB861 AB862 AB863 AB864 AB865 AB866 AB867 AB868 AB869 AB870 AB871 AB872 AB873 AB874 AB875 AB876 AB877 AB878 AB879 AB880 AB881 AB882 AB883 AB884 AB885 AB886 AB887 AB888 AB889 AB890 AB891 AB892 AB893 AB894 AB895 AB896 AB897 AB898 AB899 AB900 AB901 AB902 AB903 AB904 AB905 AB906 AB907 AB908 AB909 AB910 AB911 AB912 AB913 AB914 AB915 AB916 AB917 AB918 AB919 AB920 AB921 AB922 AB923 AB924 AB925 AB926 AB927 AB928 AB929 AB930 AB931 AB932 AB933 AB934 AB935 AB936 AB937 AB938 AB939 AB940 AB941 AB942 AB943 AB944 AB945 AB946 AB947 AB948 AB949 AB950 AB951 AB952 AB953 AB954 AB955 AB956 AB957 AB958 AB959 AB960 AB961 AB962 AB963 AB964 AB965 AB966 AB967 AB968 AB969 AB970 AB971 AB972 AB973 AB974 AB975 AB976 AB977 AB978 AB979 AB980 AB981 AB982 AB983 AB984 AB985 AB986 AB987 AB988 AB989 AB990 AB991 AB992 AB993 AB994 AB995 AB996 AB997 AB998 AB999 AB1000 AB1001 AB1002 AB1003 AB1004 AB1005 AB1006 AB1007 AB1008 AB1009 AB1010 AB1011 AB1012 AB1013 AB1014 AB1015 AB1016 AB1017 AB1018 AB1019 AB1020 AB1021 AB1022 AB1023 AB1024 AB1025 AB1026 AB1027 AB1028 AB1029 AB1030 AB1031 AB1032 AB1033 AB1034 AB1035 AB1036 AB1037 AB1038 AB1039 AB1040 AB1041 AB1042 AB1043 AB1044 AB1045 AB1046 AB1047 AB1048 AB1049 AB1050 AB1051 AB1052 AB1053 AB1054 AB1055 AB1056 AB1057 AB1058 AB1059 AB1060 AB1061 AB1062 AB1063 AB1064 AB1065 AB1066 AB1067 AB1068 AB1069 AB1070 AB1071 AB1072 AB1073 AB1074 AB1075 AB1076 AB1077 AB1078 AB1079 AB1080 AB1081 AB1082 AB1083 AB1084 AB1085 AB1086 AB1087 AB1088 AB1089 AB1090 AB1091 AB1092 AB1093 AB1094 AB1095 AB1096 AB1097 AB1098 AB1099 AB1100 AB1101 AB1102 AB1103 AB1104 AB1105 AB1106 AB1107 AB1108 AB1109 AB1110 AB1111 AB1112 AB1113 AB1114 AB1115 AB1116 AB1117 AB1118 AB1119 AB1120 AB1121 AB1122 AB1123 AB1124 AB1125 AB1126 AB1127 AB1128 AB1129 AB1130 AB1131 AB1132 AB1133 AB1134 AB1135 AB1136 AB1137 AB1138 AB1139 AB1140 AB1141 AB1142 AB1143 AB1144 AB1145 AB1146 AB1147 AB1148 AB1149 AB1150 AB1151 AB1152 AB1153 AB1154 AB1155 AB1156 AB1157 AB1158 AB1159 AB1160 AB1161 AB1162 AB1163 AB1164 AB1165 AB1166 AB1167 AB1168 AB1169 AB1170 AB1171 AB1172 AB1173 AB1174 AB1175 AB1176 AB1177 AB1178 AB1179 AB1180 AB1181 AB1182 AB1183 AB1184 AB1185 AB1186 AB1187 AB1188 AB1189 AB1190 AB1191 AB1192 AB1193 AB1194 AB1195 AB1196 AB1197 AB1198 AB1199 AB1200 AB1201 AB1202 AB1203 AB1204 AB1205 AB1206 AB1207 AB1208 AB1209 AB1210 AB1211 AB1212 AB1213 AB1214 AB1215 AB1216 AB1217 AB1218 AB1219 AB1220 AB1221 AB1222 AB1223 AB1224 AB1225 AB1226 AB1227 AB1228 AB1229 AB1230 AB1231 AB1232 AB1233 AB1234 AB1235 AB1236 AB1237 AB1238 AB1239 AB1240 AB1241 AB1242 AB1243 AB1244 AB1245 AB1246 AB1247 AB1248 AB1249 AB1250 AB1251 AB1252 AB1253 AB1254 AB1255 AB1256 AB1257 AB1258 AB1259 AB1260 AB1261 AB1262 AB1263 AB1264 AB1265 AB1266 AB1267 AB1268 AB1269 AB1270 AB1271 AB1272 AB1273 AB1274 AB1275 AB1276 AB1277 AB1278 AB1279 AB1280 AB1281 AB1282 AB1283 AB1284 AB1285 AB1286 AB1287 AB1288 AB1289 AB1290 AB1291 AB1292 AB1293 AB1294 AB1295 AB1296 AB1297 AB1298 AB1299 AB1300 AB1301 AB1302 AB1303 AB1304 AB1305 AB1306 AB1307 AB1308 AB1309 AB1310 AB1311 AB1312 AB1313 AB1314 AB1315 AB1316 AB1317 AB1318 AB1319 AB1320 AB1321 AB1322 AB1323 AB1324 AB1325 AB1326 AB1327 AB1328 AB1329 AB1330 AB1331 AB1332 AB1333 AB1334 AB1335 AB1336 AB1337 AB1338 AB1339 AB1340 AB1341 AB1342 AB1343 AB1344 AB1345 AB1346 AB1347 AB1348 AB1349 AB1350 AB1351 AB1352 AB1353 AB1354 AB1355 AB1356 AB1357 AB1358 AB1359 AB1360 AB1361 AB1362 AB1363 AB1364 AB1365 AB1366 AB1367 AB1368 AB1369 AB1370 AB1371 AB1372 AB1373 AB1374 AB1375 AB1376 AB1377 AB1378 AB1379 AB1380 AB1381 AB1382 AB1383 AB1384 AB1385 AB1386 AB1387 AB1388 AB1389 AB1390 AB1391 AB1392 AB1393 AB1394 AB1395 AB1396 AB1397 AB1398 AB1399 AB1400 AB1401 AB1402 AB1403 AB1404 AB1405 AB1406 AB1407 AB1408 AB1409 AB1410 AB1411 AB1412 AB1413 AB1414 AB1415 AB1416 AB1417 AB1418 AB1419 AB1420 AB1421 AB1422 AB1423 AB1424 AB1425 AB1426 AB1427 AB1428 AB1429 AB1430 AB1431 AB1432 AB1433 AB1434 AB1435 AB1436 AB1437 AB1438 AB1439 AB1440 AB1441 AB1442 AB1443 AB1444 AB1445 AB1446 AB1447 AB1448 AB1449 AB1450 AB1451 AB1452 AB1453 AB1454 AB1455 AB1456 AB1457 AB1458 AB1459 AB1460 AB1461 AB1462 AB1463 AB1464 AB1465 AB1466 AB1467 AB1468 AB1469 AB1470 AB1471 AB1472 AB1473 AB1474 AB1475 AB1476 AB1477 AB1478 AB1479 AB1480 AB1481 AB1482 AB1483 AB1484 AB1485 AB1486 AB1487 AB1488 AB1489 AB1490 AB1491 AB1492 AB1493 AB1494 AB1495 AB1496 AB1497 AB1498 AB1499 AB1500 AB1501 AB1502 AB1503 AB1504 AB1505 AB1506 AB1507 AB1508 AB1509 AB1510 AB1511 AB1512 AB1513 AB1514 AB1515 AB1516 AB1517 AB1518 AB1519 AB1520 AB1521 AB1522 AB1523 AB1524 AB1525 AB1526 AB1527 AB1528 AB1529 AB1530 AB1531 AB1532 AB1533 AB1534 AB1535 AB1536 AB1537 AB1538 AB1539 AB1540 AB1541 AB1542 AB1543 AB1544 AB1545 AB1546 AB1547 AB1548 AB1549 AB1550 AB1551 AB1552 AB1553 AB1554 AB1555 AB1556 AB1557 AB1558 AB1559 AB1560 AB1561 AB1562 AB1563 AB1564 AB1565 AB1566 AB1567 AB1568 AB1569 AB1570 AB1571 AB1572 AB1573 AB1574 AB1575 AB1576 AB1577 AB1578 AB1579 AB1580 AB1581 AB1582 AB1583 AB1584 AB1585 AB1586 AB1587 AB1588 AB1589 AB1590 AB1591 AB1592 AB1593 AB1594 AB1595 AB1596 AB1597 AB1598 AB1599 AB1600 AB1601 AB1602 AB1603 AB1604 AB1605 AB1606 AB1607 AB1608 AB1609 AB1610 AB1611 AB1612 AB1613 AB1614 AB1615 AB1616 AB1617 AB1618 AB1619 AB1620 AB1621 AB1622 AB1623 AB1624 AB1625 AB1626 AB1627 AB1628 AB1629 AB1630 AB1631 AB1632 AB1633 AB1634 AB1635 AB1636 AB1637 AB1638 AB1639 AB1640 AB1641 AB1642 AB1643 AB1644 AB1645 AB1646 AB1647 AB1648 AB1649 AB1650 AB1651 AB1652 AB1653 AB1654 AB1655 AB1656 AB1657 AB1658 AB1659 AB1660 AB1661 AB1662 AB1663 AB1664 AB1665 AB1666 AB1667 AB1668 AB1669 AB1670 AB1671 AB1672 AB1673 AB1674 AB1675 AB1676 AB1677 AB1678 AB1679 AB1680 AB1681 AB1682 AB1683 AB1684 AB1685 AB1686 AB1687 AB1688 AB1689 AB1690 AB1691 AB1692 AB1693 AB1694 AB1695 AB1696 AB1697 AB1698 AB1699 AB1700 AB1701 AB1702 AB1703 AB1704 AB1705 AB1706 AB1707 AB1708 AB1709 AB1710 AB1711 AB1712 AB1713 AB1714 AB1715 AB1716 AB1717 AB1718 AB1719 AB1720 AB1721 AB1722 AB1723 AB1724 AB1725 AB1726 AB1727 AB1728 AB1729 AB1730 AB1731 AB1732 AB1733 AB1734 AB1735 AB1736 AB1737 AB1738 AB1739 AB1740 AB1741 AB1742 AB1743 AB1744 AB1745 AB1746 AB1747 AB1748 AB1749 AB1750 AB1751 AB1752 AB1753 AB1754 AB1755 AB1756 AB1757 AB1758 AB1759 AB1760 AB1761 AB1762 AB1763 AB1764 AB1765 AB1766 AB1767 AB1768 AB1769 AB1770 AB1771 AB1772 AB1773 AB1774 AB1775 AB1776 AB1777 AB1778 AB1779 AB1780 AB1781 AB1782 AB1783 AB1784 AB1785 AB1786 AB1787 AB1788 AB1789 AB1790 AB1791 AB1792 AB1793 AB1794 AB1795 AB1796 AB1797 AB1798 AB1799 AB1800 AB1801 AB1802 AB1803 AB1804 AB1805 AB1806 AB1807 AB1808 AB1809 AB1810 AB1811 AB1812 AB1813 AB1814 AB1815 AB1816 AB1817 AB1818 AB1819 AB1820 AB1821 AB1822 AB1823 AB1824 AB1825 AB1826 AB1827 AB1828 AB1829 AB1830 AB1831 AB1832 AB1833 AB1834 AB1835 AB1836 AB1837 AB1838 AB1839 AB1840 AB1841 AB1842 AB1843 AB1844 AB1845 AB1846 AB1847 AB1848 AB1849 AB1850 AB1851 AB1852 AB1853 AB1854 AB1855 AB1856 AB1857 AB1858 AB1859 AB1860 AB1861 AB1862 AB1863 AB1864 AB1865 AB1866 AB1867 AB1868 AB1869 AB1870 AB1871 AB1872 AB1873 AB1874 AB1875 AB1876 AB1877 AB1878 AB1879 AB1880 AB1881 AB1882 AB1883 AB1884 AB1885 AB1886 AB1887 AB1888 AB1889 AB1890 AB1891 AB1892 AB1893 AB1894 AB1895 AB1896 AB1897 AB1898 AB1899 AB1900 AB1901 AB1902 AB1903 AB1904 AB1905 AB1906 AB1907 AB1908 AB1909 AB1910 AB1911 AB1912 AB1913 AB1914 AB1915 AB1916 AB1917 AB1918 AB1919 AB1920 AB1921 AB1922 AB1923 AB1924 AB1925 AB1926 AB1927 AB1928 AB1929 AB1930 AB1931 AB1932 AB1933 AB1934 AB1935 AB1936 AB1937 AB1938 AB1939 AB1940 AB1941 AB1942 AB1943 AB1944 AB1945 AB1946 AB1947 AB1948 AB1949 AB1950 AB1951 AB1952 AB1953 AB1954 AB1955 AB1956 AB1957 AB1958 AB1959 AB1960 AB1961 AB1962 AB1963 AB1964 AB1965 AB1966 AB1967 AB1968 AB1969 AB1970 AB1971 AB1972 AB1973 AB1974 AB1975 AB1976 AB1977 AB1978 AB1979 AB1980 AB1981 AB1982 AB1983 AB1984 AB1985 AB1986 AB1987 AB1988 AB1989 AB1990 AB1991 AB1992 AB1993 AB1994 AB1995 AB1996 AB1997" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="date" operator="greaterThanOrEqual">
       <formula1>DATE(2000,1,1)</formula1>
+    </dataValidation>
+    <dataValidation sqref="AE8:AE2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Status</formula1>
     </dataValidation>
     <dataValidation sqref="K8:K2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Objekt_Einordnung</formula1>
     </dataValidation>
-    <dataValidation sqref="AE8:AE2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Status</formula1>
+    <dataValidation sqref="L8:L2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Klassen_Zuordnung</formula1>
+    </dataValidation>
+    <dataValidation sqref="M8:M2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Affectation_de_classe</formula1>
+    </dataValidation>
+    <dataValidation sqref="N8:N2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Assegnazione_della_classe</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7086614173228347" right="0.7086614173228347" top="0.7874015748031497" bottom="0.7874015748031497" header="0.3149606299212598" footer="0.3149606299212598"/>
@@ -24567,7 +24141,7 @@
     <row r="357" ht="13.5" customHeight="1" s="223"/>
   </sheetData>
   <autoFilter ref="A2:V60"/>
-  <dataValidations count="6">
+  <dataValidations count="9">
     <dataValidation sqref="AC8:AC2000" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Versionsdatum" prompt="Datum im Format YYYY-MM-DD eintragen." type="date">
       <formula1>DATE(2000,1,1)</formula1>
       <formula2>DATE(2100,12,31)</formula2>
@@ -24585,7 +24159,16 @@
       <formula1>Status</formula1>
     </dataValidation>
     <dataValidation sqref="G8:G2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Property-Assignment</formula1>
+      <formula1>Property_Classification</formula1>
+    </dataValidation>
+    <dataValidation sqref="H8:H2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Merkmals_Zuordnung</formula1>
+    </dataValidation>
+    <dataValidation sqref="I8:I2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Attribution_de_propriete</formula1>
+    </dataValidation>
+    <dataValidation sqref="J8:J2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>Assegnazione_della_proprieta</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7086614173228347" right="0.7086614173228347" top="0.7874015748031497" bottom="0.7874015748031497" header="0.3149606299212598" footer="0.3149606299212598"/>

</xml_diff>